<commit_message>
Restore DQN baseline and verified experiment evidence
</commit_message>
<xml_diff>
--- a/output/excel/pareto_metrics_10_130.xlsx
+++ b/output/excel/pareto_metrics_10_130.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="17">
   <si>
     <t>Config</t>
   </si>
@@ -62,6 +62,9 @@
   </si>
   <si>
     <t>PSP</t>
+  </si>
+  <si>
+    <t>DQN</t>
   </si>
 </sst>
 </file>
@@ -419,7 +422,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
@@ -465,19 +468,19 @@
         <v>12</v>
       </c>
       <c r="C2">
-        <v>0.8190858049530542</v>
+        <v>0.8313320455316456</v>
       </c>
       <c r="D2">
-        <v>0.07845943299876014</v>
+        <v>0.07716094725795759</v>
       </c>
       <c r="E2">
-        <v>0.01123303647156375</v>
+        <v>0.01106219628949759</v>
       </c>
       <c r="F2">
-        <v>0.3894061417240519</v>
+        <v>0.3807984459227371</v>
       </c>
       <c r="G2">
-        <v>0.3894061417240519</v>
+        <v>0.3807984459227371</v>
       </c>
       <c r="H2">
         <v>50</v>
@@ -486,7 +489,7 @@
         <v>50</v>
       </c>
       <c r="J2">
-        <v>0.01156692475120008</v>
+        <v>0.01107531228391787</v>
       </c>
       <c r="K2">
         <v>0.09343455008250155</v>
@@ -500,19 +503,19 @@
         <v>13</v>
       </c>
       <c r="C3">
-        <v>0.8596083232861803</v>
+        <v>0.8698059002848453</v>
       </c>
       <c r="D3">
-        <v>0.04924774922905724</v>
+        <v>0.04813224535102884</v>
       </c>
       <c r="E3">
-        <v>0.007909548101354831</v>
+        <v>0.00763933705929001</v>
       </c>
       <c r="F3">
-        <v>0.3550407681321283</v>
+        <v>0.3460106877058775</v>
       </c>
       <c r="G3">
-        <v>0.3550407681321283</v>
+        <v>0.3460106877058775</v>
       </c>
       <c r="H3">
         <v>50</v>
@@ -521,7 +524,7 @@
         <v>50</v>
       </c>
       <c r="J3">
-        <v>0.03118206734034162</v>
+        <v>0.02985678050828587</v>
       </c>
       <c r="K3">
         <v>0.1004159586707601</v>
@@ -535,19 +538,19 @@
         <v>14</v>
       </c>
       <c r="C4">
-        <v>0.8945274818380959</v>
+        <v>0.9064394470271963</v>
       </c>
       <c r="D4">
-        <v>0.03264358629038765</v>
+        <v>0.03175369102684482</v>
       </c>
       <c r="E4">
-        <v>0.004473083981186269</v>
+        <v>0.004318919542992977</v>
       </c>
       <c r="F4">
-        <v>0.3362910219633266</v>
+        <v>0.3263379571657256</v>
       </c>
       <c r="G4">
-        <v>0.3362910219633266</v>
+        <v>0.3263379571657256</v>
       </c>
       <c r="H4">
         <v>50</v>
@@ -556,7 +559,7 @@
         <v>50</v>
       </c>
       <c r="J4">
-        <v>0.06476404001480258</v>
+        <v>0.06201146660504325</v>
       </c>
       <c r="K4">
         <v>0.03200121896407809</v>
@@ -570,19 +573,19 @@
         <v>15</v>
       </c>
       <c r="C5">
-        <v>0.9470099455117535</v>
+        <v>0.9581874358420364</v>
       </c>
       <c r="D5">
-        <v>0.001610733781728429</v>
+        <v>0.001592270780686548</v>
       </c>
       <c r="E5">
-        <v>0.01083021880625903</v>
+        <v>0.01068470524612985</v>
       </c>
       <c r="F5">
-        <v>0.3281985745086926</v>
+        <v>0.3184655491881143</v>
       </c>
       <c r="G5">
-        <v>0.3281985745086926</v>
+        <v>0.3184655491881143</v>
       </c>
       <c r="H5">
         <v>50</v>
@@ -595,6 +598,41 @@
       </c>
       <c r="K5">
         <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6">
+        <v>0.3381908168404409</v>
+      </c>
+      <c r="D6">
+        <v>0.4048305563171643</v>
+      </c>
+      <c r="E6">
+        <v>0.009723489810460728</v>
+      </c>
+      <c r="F6">
+        <v>0.5973779158170724</v>
+      </c>
+      <c r="G6">
+        <v>0.5973779158170724</v>
+      </c>
+      <c r="H6">
+        <v>4</v>
+      </c>
+      <c r="I6">
+        <v>5</v>
+      </c>
+      <c r="J6">
+        <v>0.3927574576977676</v>
+      </c>
+      <c r="K6">
+        <v>0.43389371206371</v>
       </c>
     </row>
   </sheetData>

</xml_diff>